<commit_message>
OBS-0016 vuelve a discusión: la fecha aproximada se retiró con DEC-206
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Versión 6 · Validación DGIVA</t>
+          <t>Versión 15 · Validación DGIVA</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tabla 1. Observaciones registradas en la hoja de revisión, decisión de la Secretaría y texto vigente en la versión 5.</t>
+          <t>Tabla 1. Observaciones registradas en la hoja de revisión, decisión de la Secretaría y texto vigente en la versión 15.</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       <c r="J20" s="21" t="n"/>
       <c r="K20" s="21" t="n"/>
     </row>
-    <row r="21" ht="39" customHeight="1">
+    <row r="21" ht="78" customHeight="1">
       <c r="A21" s="22" t="inlineStr">
         <is>
           <t>OBS-0016</t>
@@ -1756,22 +1756,22 @@
       </c>
       <c r="F21" s="24" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>En discusión</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>La fecha ya era opcional; ahora todos los campos no obligatorios dicen «(opcional)». Además, la casilla «No sé la fecha exacta» permite indicar mes y año aproximados.</t>
+          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»: con «Sí» se pide la fecha exacta; con «No» no se pide ninguna. Se retiraron la casilla «No sé la fecha exacta» y el mes y año aproximados, de modo que ya no se registra una fecha aproximada. Pregunta para la DGIVA: ¿basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>DEC-191</t>
+          <t>DEC-191, DEC-206</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">
         <is>
-          <t>Atendida</t>
+          <t>Para discusión</t>
         </is>
       </c>
       <c r="J21" s="21" t="n"/>
@@ -2564,7 +2564,7 @@
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Fuente: hoja «Revisión · Formulario de Denuncia Ambiental» (modo revisión del formulario) y documento 05 «Decisiones y pendientes», DEC-188 a DEC-196. Nota: las columnas en color crema son para llenado de la DGIVA.</t>
+          <t>Fuente: hoja «Revisión · Formulario de Denuncia Ambiental» (modo revisión del formulario) y documento 05 «Decisiones y pendientes», DEC-188 a DEC-210. Nota: las columnas en color crema son para llenado de la DGIVA.</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2756,22 +2756,22 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>OBS-0020</t>
+          <t>OBS-0016</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Casos de otra autoridad</t>
+          <t>Fecha aproximada</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>¿Qué autoridad atiende el arbolado en vía pública y los hechos dentro de viviendas, condominios o unidades habitacionales? ¿Qué casos de arbolado sí atiende la Secretaría?</t>
+          <t>¿Basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>El formulario tiene la tarjeta «Daño a arbolado urbano» como competencia de la Secretaría; en 2026, el 40.7 % de las denuncias de arbolado se declararon incompetencia.</t>
+          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»; con «No» no se pide fecha y ya no se registra una aproximada, que era lo que pedía la observación.</t>
         </is>
       </c>
       <c r="F9" s="21" t="n"/>
@@ -2782,22 +2782,22 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>P-09</t>
+          <t>OBS-0020</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Datos de la DGCORENADR</t>
+          <t>Casos de otra autoridad</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
+          <t>¿Qué autoridad atiende el arbolado en vía pública y los hechos dentro de viviendas, condominios o unidades habitacionales? ¿Qué casos de arbolado sí atiende la Secretaría?</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
+          <t>El formulario tiene la tarjeta «Daño a arbolado urbano» como competencia de la Secretaría; en 2026, el 40.7 % de las denuncias de arbolado se declararon incompetencia.</t>
         </is>
       </c>
       <c r="F10" s="21" t="n"/>
@@ -2808,28 +2808,54 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
+          <t>P-09</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Datos de la DGCORENADR</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
           <t>P-07</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>Plazo para informar</t>
         </is>
       </c>
-      <c r="D11" s="27" t="inlineStr">
+      <c r="D12" s="26" t="inlineStr">
         <is>
           <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
         </is>
       </c>
-      <c r="F11" s="21" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="F12" s="21" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Nota: P-07 y P-09 son preguntas abiertas del documento 05 del proyecto; las demás derivan de observaciones de la revisión. La columna en color crema es para llenado de la DGIVA.</t>
         </is>
@@ -2837,8 +2863,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.6" right="0.6" top="0.7" bottom="0.7" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
La fecha admite ser aproximada; Versión 16 (DEC-211)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -1728,7 +1728,7 @@
       <c r="J20" s="21" t="n"/>
       <c r="K20" s="21" t="n"/>
     </row>
-    <row r="21" ht="78" customHeight="1">
+    <row r="21" ht="104" customHeight="1">
       <c r="A21" s="22" t="inlineStr">
         <is>
           <t>OBS-0016</t>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»: con «Sí» se pide la fecha exacta; con «No» no se pide ninguna. Se retiraron la casilla «No sé la fecha exacta» y el mes y año aproximados, de modo que ya no se registra una fecha aproximada. Pregunta para la DGIVA: ¿basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
+          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»: con «Sí» se pide la fecha exacta; con «No» no se pide ninguna. Se retiraron la casilla «No sé la fecha exacta» y el mes y año aproximados, de modo que ya no se registra una fecha aproximada. Desde DEC-211 la ayuda de la fecha dice que puede ser aproximada, de modo que quien no la sabe con exactitud contesta «Sí» y elige un día cercano. Pregunta para la DGIVA: ¿basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>DEC-191, DEC-206</t>
+          <t>DEC-191, DEC-206, DEC-211</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Textos simplificados en todo el formulario; Versión 25
DEC-220: fuera las ayudas que explican el propósito interno del dato, los
«déjalo en blanco» en campos opcionales y los avisos que repiten la ayuda;
textos más cortos en portada, pasos 1 a 6 y acuse. La hoja de control
registra el cambio en OBS-0007, OBS-0018 y OBS-0019.
DEC-221: al abrir la fase 2 se pasa a Claude Code; hasta entonces el envío
sigue siendo manual.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Versión 24 · Validación DGIVA</t>
+          <t>Versión 25 · Validación DGIVA</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       <c r="J11" s="21" t="n"/>
       <c r="K11" s="21" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="39" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
           <t>OBS-0007</t>
@@ -1320,12 +1320,12 @@
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>Dice ahora «La ubicación determina qué unidad administrativa competente la atiende». También se atiende OBS-0018.</t>
+          <t>Dice ahora «La ubicación determina qué unidad administrativa competente la atiende». También se atiende OBS-0018. Después, al simplificar los textos (DEC-220), se retiró esa viñeta: era proceso interno.</t>
         </is>
       </c>
       <c r="H12" s="20" t="inlineStr">
         <is>
-          <t>DEC-188</t>
+          <t>DEC-188, DEC-220</t>
         </is>
       </c>
       <c r="I12" s="20" t="inlineStr">
@@ -1826,7 +1826,7 @@
       <c r="J22" s="21" t="n"/>
       <c r="K22" s="21" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="52" customHeight="1">
       <c r="A23" s="22" t="inlineStr">
         <is>
           <t>OBS-0018</t>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="G23" s="23" t="inlineStr">
         <is>
-          <t>Dice ahora «unidad administrativa competente» en lugar de «oficina». Se atiende junto con OBS-0007.</t>
+          <t>Dice ahora «unidad administrativa competente» en lugar de «oficina». Se atiende junto con OBS-0007. Después, al simplificar los textos (DEC-220), los dos textos que decían «unidad administrativa» se retiraron; en ningún lugar se dice «oficina».</t>
         </is>
       </c>
       <c r="H23" s="24" t="inlineStr">
         <is>
-          <t>DEC-188</t>
+          <t>DEC-188, DEC-220</t>
         </is>
       </c>
       <c r="I23" s="24" t="inlineStr">
@@ -1875,7 +1875,7 @@
       <c r="J23" s="21" t="n"/>
       <c r="K23" s="21" t="n"/>
     </row>
-    <row r="24" ht="78" customHeight="1">
+    <row r="24" ht="104" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
           <t>OBS-0019</t>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="G24" s="19" t="inlineStr">
         <is>
-          <t>Se incorporó el contenido de la propuesta, en el registro de «tú» que usa todo el formulario: la Secretaría valora los hechos con el mismo rigor y el correo sirve para que la unidad administrativa que atiende la denuncia pueda ponerse en contacto. No se incluye el envío del informe de acciones por correo, porque el formulario no envía correos y no hay un plazo comprometido para informar.</t>
+          <t>Se incorporó el contenido de la propuesta, en el registro de «tú» que usa todo el formulario: la Secretaría valora los hechos con el mismo rigor y el correo sirve para que la unidad administrativa que atiende la denuncia pueda ponerse en contacto. No se incluye el envío del informe de acciones por correo, porque el formulario no envía correos y no hay un plazo comprometido para informar. Después se simplificó (DEC-220): «Sí. Al final eliges presentarla anónima; sólo te pedimos un correo por si hay que aclarar algo. Se atiende con el mismo rigor.».</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
         <is>
-          <t>DEC-195</t>
+          <t>DEC-195, DEC-220</t>
         </is>
       </c>
       <c r="I24" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Respuestas de la reunión con la DGIVA: fuera olores y anuncios; Versión 26
DEC-222: olores y anuncios o luz excesiva salen de «Mi caso no está en la
lista» y no se mencionan. OBS-0016 atendida tal como está; el arbolado
urbano es de la DGIVA (OBS-0020, queda viviendas y condominios); el
teléfono sigue obligatorio (P-17).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Versión 25 · Validación DGIVA</t>
+          <t>Versión 26 · Validación DGIVA</t>
         </is>
       </c>
     </row>
@@ -1173,17 +1173,17 @@
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>Aplicado con lo que confirmó la DGIVA: la tarjeta queda «Ruido o vibraciones · De una industria o fábrica» y salen olores, anuncios, luz excesiva y «de un negocio». El ruido de comercios, bares, restaurantes y salones se orienta al INVEA en «Mi caso no está en la lista». Pregunta para la DGIVA: olores, anuncios y luz excesiva también pasaron a esa lista con la PAOT como instancia receptora; ¿es la instancia correcta?</t>
+          <t>Aplicado con lo que confirmó la DGIVA: la tarjeta queda «Ruido o vibraciones · De una industria o fábrica» y salen olores, anuncios, luz excesiva y «de un negocio». El ruido de comercios, bares, restaurantes y salones se orienta al INVEA en «Mi caso no está en la lista». Olores, anuncios y luz excesiva tampoco se orientan a otra autoridad: no hay norma aplicable que permita decir a dónde acudir, y el formulario no los menciona (decisión del 20 oct 2026).</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
-          <t>DEC-190 (en parte)</t>
+          <t>DEC-190, DEC-222</t>
         </is>
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
-          <t>Para discusión</t>
+          <t>Atendida</t>
         </is>
       </c>
       <c r="J9" s="21" t="n"/>
@@ -1728,7 +1728,7 @@
       <c r="J20" s="21" t="n"/>
       <c r="K20" s="21" t="n"/>
     </row>
-    <row r="21" ht="104" customHeight="1">
+    <row r="21" ht="39" customHeight="1">
       <c r="A21" s="22" t="inlineStr">
         <is>
           <t>OBS-0016</t>
@@ -1761,17 +1761,17 @@
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»: con «Sí» se pide la fecha exacta; con «No» no se pide ninguna. Se retiraron la casilla «No sé la fecha exacta» y el mes y año aproximados, de modo que ya no se registra una fecha aproximada. Desde DEC-211 la ayuda de la fecha dice que puede ser aproximada, de modo que quien no la sabe con exactitud contesta «Sí» y elige un día cercano. Pregunta para la DGIVA: ¿basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
+          <t>El formulario pregunta «¿Conoces la fecha en que ocurrió o inició?» (DEC-206): con «Sí» se pide la fecha y la ayuda dice que puede ser aproximada (DEC-211); con «No» no se pide ninguna. Se confirmó el 20 oct 2026 que basta así.</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>DEC-191, DEC-206, DEC-211</t>
+          <t>DEC-191, DEC-206, DEC-211, DEC-222</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">
         <is>
-          <t>Para discusión</t>
+          <t>Atendida</t>
         </is>
       </c>
       <c r="J21" s="21" t="n"/>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Para no mencionar casos que no aparecen en «Mi caso no está en la lista», la respuesta conserva los ejemplos que ya existen ahí. Preguntas para la DGIVA: ¿qué autoridad atiende el arbolado en vía pública y los hechos dentro de viviendas, condominios o unidades habitacionales? ¿Qué casos de arbolado sí atiende la Secretaría?</t>
+          <t>Arbolado: la DGIVA atiende todo el arbolado urbano en suelo urbano y en las áreas de valor ambiental, de modo que no se orienta a otra autoridad; el formulario ya lo trata como competencia de la Secretaría (20 oct 2026). Queda la pregunta: ¿qué autoridad atiende los hechos dentro de viviendas, condominios o unidades habitacionales?</t>
         </is>
       </c>
       <c r="H25" s="24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEC-222</t>
         </is>
       </c>
       <c r="I25" s="24" t="inlineStr">
@@ -2607,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2678,74 +2678,74 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>OBS-0004</t>
+          <t>OBS-0027</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Instancia para olores, anuncios y luz</t>
+          <t>Caso de Los Dinamos</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>¿La PAOT es la instancia correcta para orientar las denuncias de malos olores y de anuncios o luz excesiva?</t>
+          <t>¿Coinciden en turnar a la DGCORENADR el caso del restaurante en Los Dinamos? ¿Quién atiende el uso de leña sin legal procedencia?</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Esos supuestos salieron de la tarjeta de ruido y ahora aparecen en «Mi caso no está en la lista» remitiendo a la PAOT.</t>
+          <t>Con el cruce espacial del formulario, el punto cae en suelo de conservación (La Magdalena Contreras).</t>
         </is>
       </c>
       <c r="F6" s="21" t="n"/>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="117" customHeight="1">
       <c r="A7" s="24" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>OBS-0027</t>
+          <t>OBS-0024</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Caso de Los Dinamos</t>
+          <t>Giros fuera de competencia</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>¿Coinciden en turnar a la DGCORENADR el caso del restaurante en Los Dinamos? ¿Quién atiende el uso de leña sin legal procedencia?</t>
+          <t>¿Qué giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>Con el cruce espacial del formulario, el punto cae en suelo de conservación (La Magdalena Contreras).</t>
+          <t>Lista actual: obra en construcción o demolición; taller mecánico, hojalatería o pintura; industria o fábrica; bodega o almacén; restaurante, fonda o cocina económica; bar, cantina, salón de fiestas o antro; tienda, abarrotes u otro comercio; panadería o tortillería; carnicería, pollería o pescadería; lavandería o tintorería; gasolinera o estación de servicio; estacionamiento o pensión; hospital, clínica, consultorio o laboratorio; escuela, oficina o edificio público; banco de materiales, mina o tiro de tierra; centro de acopio o reciclaje; vivero, granja, establo o rastro; espectáculo público, feria o evento; otro.</t>
         </is>
       </c>
       <c r="F7" s="21" t="n"/>
     </row>
-    <row r="8" ht="117" customHeight="1">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="20" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>OBS-0024</t>
+          <t>OBS-0020</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Giros fuera de competencia</t>
+          <t>Viviendas, condominios y unidades habitacionales</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>¿Qué giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
+          <t>¿Qué autoridad atiende los hechos que ocurren dentro de viviendas, condominios o unidades habitacionales?</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Lista actual: obra en construcción o demolición; taller mecánico, hojalatería o pintura; industria o fábrica; bodega o almacén; restaurante, fonda o cocina económica; bar, cantina, salón de fiestas o antro; tienda, abarrotes u otro comercio; panadería o tortillería; carnicería, pollería o pescadería; lavandería o tintorería; gasolinera o estación de servicio; estacionamiento o pensión; hospital, clínica, consultorio o laboratorio; escuela, oficina o edificio público; banco de materiales, mina o tiro de tierra; centro de acopio o reciclaje; vivero, granja, establo o rastro; espectáculo público, feria o evento; otro.</t>
+          <t>El arbolado ya está resuelto: la DGIVA atiende todo el arbolado urbano en suelo urbano y en las áreas de valor ambiental (20 oct 2026), y el formulario lo trata como competencia de la Secretaría.</t>
         </is>
       </c>
       <c r="F8" s="21" t="n"/>
@@ -2756,22 +2756,22 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>OBS-0016</t>
+          <t>P-09</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Fecha aproximada</t>
+          <t>Datos de la DGCORENADR</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>¿Basta con registrar que la persona no conoce la fecha, o se necesita una fecha aproximada (mes y año)?</t>
+          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Desde DEC-206 el formulario pregunta «¿Conoces la fecha en que ocurrió o inició?»; con «No» no se pide fecha y ya no se registra una aproximada, que era lo que pedía la observación.</t>
+          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
         </is>
       </c>
       <c r="F9" s="21" t="n"/>
@@ -2782,80 +2782,28 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>OBS-0020</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Casos de otra autoridad</t>
+          <t>Plazo para informar</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>¿Qué autoridad atiende el arbolado en vía pública y los hechos dentro de viviendas, condominios o unidades habitacionales? ¿Qué casos de arbolado sí atiende la Secretaría?</t>
+          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>El formulario tiene la tarjeta «Daño a arbolado urbano» como competencia de la Secretaría; en 2026, el 40.7 % de las denuncias de arbolado se declararon incompetencia.</t>
+          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
         </is>
       </c>
       <c r="F10" s="21" t="n"/>
     </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>P-09</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>Datos de la DGCORENADR</t>
-        </is>
-      </c>
-      <c r="D11" s="27" t="inlineStr">
-        <is>
-          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
-        </is>
-      </c>
-      <c r="F11" s="21" t="n"/>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>P-07</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Plazo para informar</t>
-        </is>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
-        </is>
-      </c>
-      <c r="F12" s="21" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="25" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Nota: P-07 y P-09 son preguntas abiertas del documento 05 del proyecto; las demás derivan de observaciones de la revisión. La columna en color crema es para llenado de la DGIVA.</t>
         </is>
@@ -2864,8 +2812,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.6" right="0.6" top="0.7" bottom="0.7" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
OBS-0020 atendida: viviendas, condominios y vía pública los recibe la Secretaría
DEC-223: la DGIVA recibe, inspecciona y, si corresponde, deriva a la
alcaldía; construcción, siempre la DGIVA. El formulario no cambia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -1924,7 +1924,7 @@
       <c r="J24" s="21" t="n"/>
       <c r="K24" s="21" t="n"/>
     </row>
-    <row r="25" ht="65" customHeight="1">
+    <row r="25" ht="91" customHeight="1">
       <c r="A25" s="22" t="inlineStr">
         <is>
           <t>OBS-0020</t>
@@ -1957,17 +1957,17 @@
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Arbolado: la DGIVA atiende todo el arbolado urbano en suelo urbano y en las áreas de valor ambiental, de modo que no se orienta a otra autoridad; el formulario ya lo trata como competencia de la Secretaría (20 oct 2026). Queda la pregunta: ¿qué autoridad atiende los hechos dentro de viviendas, condominios o unidades habitacionales?</t>
+          <t>No se agregan casos a «Mi caso no está en la lista». La DGIVA atiende todo el arbolado urbano en suelo urbano y en las áreas de valor ambiental. En viviendas, condominios, unidades habitacionales y vía pública, la DGIVA recibe la denuncia, realiza la inspección y, cuando el caso es de la alcaldía, se lo deriva; lo relacionado con construcción lo atiende siempre la DGIVA. Por eso el formulario recibe esos casos como competencia de la Secretaría (respuesta del 20 oct 2026).</t>
         </is>
       </c>
       <c r="H25" s="24" t="inlineStr">
         <is>
-          <t>DEC-222</t>
+          <t>DEC-222, DEC-223</t>
         </is>
       </c>
       <c r="I25" s="24" t="inlineStr">
         <is>
-          <t>Para discusión</t>
+          <t>Atendida</t>
         </is>
       </c>
       <c r="J25" s="21" t="n"/>
@@ -2607,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2730,22 +2730,22 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>OBS-0020</t>
+          <t>P-09</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Viviendas, condominios y unidades habitacionales</t>
+          <t>Datos de la DGCORENADR</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>¿Qué autoridad atiende los hechos que ocurren dentro de viviendas, condominios o unidades habitacionales?</t>
+          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>El arbolado ya está resuelto: la DGIVA atiende todo el arbolado urbano en suelo urbano y en las áreas de valor ambiental (20 oct 2026), y el formulario lo trata como competencia de la Secretaría.</t>
+          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
         </is>
       </c>
       <c r="F8" s="21" t="n"/>
@@ -2756,54 +2756,28 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>P-09</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Datos de la DGCORENADR</t>
+          <t>Plazo para informar</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
+          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
+          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
         </is>
       </c>
       <c r="F9" s="21" t="n"/>
     </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>P-07</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Plazo para informar</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
-        </is>
-      </c>
-      <c r="F10" s="21" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Nota: P-07 y P-09 son preguntas abiertas del documento 05 del proyecto; las demás derivan de observaciones de la revisión. La columna en color crema es para llenado de la DGIVA.</t>
         </is>
@@ -2812,8 +2786,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.6" right="0.6" top="0.7" bottom="0.7" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Fuera «antro», OBS-0027 atendida y pendientes consolidados; Versión 28
DEC-225: «Bar, cantina o salón de fiestas» sin «antro» (materia del
INVEA); Los Dinamos se turna a la DGCORENADR; P-20 resuelta; P-19
consolidada en P-02.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Versión 27 · Validación DGIVA</t>
+          <t>Versión 28 · Validación DGIVA</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       <c r="J28" s="21" t="n"/>
       <c r="K28" s="21" t="n"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="39" customHeight="1">
       <c r="A29" s="22" t="inlineStr">
         <is>
           <t>OBS-0024</t>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>Se retirará «antro». Pregunta para la DGIVA: ¿qué otros giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
+          <t>Se retiró «antro» de la lista de tipos de establecimiento: su funcionamiento es materia del INVEA (DEC-225). Pregunta para la DGIVA: ¿qué otros giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEC-225</t>
         </is>
       </c>
       <c r="I29" s="24" t="inlineStr">
@@ -2267,7 +2267,7 @@
       <c r="J31" s="21" t="n"/>
       <c r="K31" s="21" t="n"/>
     </row>
-    <row r="32" ht="65" customHeight="1">
+    <row r="32" ht="39" customHeight="1">
       <c r="A32" s="18" t="inlineStr">
         <is>
           <t>OBS-0027</t>
@@ -2300,17 +2300,17 @@
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
-          <t>Se retiró la pregunta sobre permisos o autorizaciones. Sobre el ejemplo del restaurante en Los Dinamos: con el cruce espacial del formulario el punto cae en suelo de conservación (La Magdalena Contreras), por lo que la denuncia se turna a la DGCORENADR. Preguntas para la DGIVA: ¿coincide con su criterio? y ¿quién atiende el uso de leña sin legal procedencia?</t>
+          <t>Se retiró la pregunta sobre permisos o autorizaciones. El caso del restaurante en Los Dinamos se turna a la DGCORENADR, como hace el cruce espacial del formulario: el punto cae en suelo de conservación (confirmado el 20 oct 2026).</t>
         </is>
       </c>
       <c r="H32" s="20" t="inlineStr">
         <is>
-          <t>DEC-191 (en parte)</t>
+          <t>DEC-191 (en parte), DEC-225</t>
         </is>
       </c>
       <c r="I32" s="20" t="inlineStr">
         <is>
-          <t>Para discusión</t>
+          <t>Atendida</t>
         </is>
       </c>
       <c r="J32" s="21" t="n"/>
@@ -2607,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2672,54 +2672,54 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="130" customHeight="1">
       <c r="A6" s="20" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>OBS-0027</t>
+          <t>OBS-0024</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Caso de Los Dinamos</t>
+          <t>Giros fuera de competencia</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>¿Coinciden en turnar a la DGCORENADR el caso del restaurante en Los Dinamos? ¿Quién atiende el uso de leña sin legal procedencia?</t>
+          <t>¿Qué giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Con el cruce espacial del formulario, el punto cae en suelo de conservación (La Magdalena Contreras).</t>
+          <t>Lista actual: obra en construcción o demolición; taller mecánico, hojalatería o pintura; industria o fábrica; bodega o almacén; restaurante, fonda o cocina económica; bar, cantina o salón de fiestas («antro» ya se retiró); tienda, abarrotes u otro comercio; panadería o tortillería; carnicería, pollería o pescadería; lavandería o tintorería; gasolinera o estación de servicio; estacionamiento o pensión; hospital, clínica, consultorio o laboratorio; escuela, oficina o edificio público; banco de materiales, mina o tiro de tierra; centro de acopio o reciclaje; vivero, granja, establo o rastro; espectáculo público, feria o evento; otro.</t>
         </is>
       </c>
       <c r="F6" s="21" t="n"/>
     </row>
-    <row r="7" ht="117" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="24" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>OBS-0024</t>
+          <t>P-09</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Giros fuera de competencia</t>
+          <t>Datos de la DGCORENADR</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>¿Qué giros de la lista «Tipo de establecimiento» quedan fuera de la competencia de la CIVASU?</t>
+          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>Lista actual: obra en construcción o demolición; taller mecánico, hojalatería o pintura; industria o fábrica; bodega o almacén; restaurante, fonda o cocina económica; bar, cantina, salón de fiestas o antro; tienda, abarrotes u otro comercio; panadería o tortillería; carnicería, pollería o pescadería; lavandería o tintorería; gasolinera o estación de servicio; estacionamiento o pensión; hospital, clínica, consultorio o laboratorio; escuela, oficina o edificio público; banco de materiales, mina o tiro de tierra; centro de acopio o reciclaje; vivero, granja, establo o rastro; espectáculo público, feria o evento; otro.</t>
+          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
         </is>
       </c>
       <c r="F7" s="21" t="n"/>
@@ -2730,54 +2730,28 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>P-09</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Datos de la DGCORENADR</t>
+          <t>Plazo para informar</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>Domicilio, horario de atención y teléfono de la Coordinación de Inspección Ambiental en Suelo de Conservación y Áreas Naturales Protegidas (DGCORENADR).</t>
+          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>La tarjeta «Presencial» los muestra todavía como «por confirmar».</t>
+          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
         </is>
       </c>
       <c r="F8" s="21" t="n"/>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>P-07</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>Plazo para informar</t>
-        </is>
-      </c>
-      <c r="D9" s="27" t="inlineStr">
-        <is>
-          <t>¿En cuántos días hábiles se responde a quien consulta el estado de su denuncia?</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>El Manual Administrativo fija los plazos del procedimiento, pero no el de informar a la persona denunciante.</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Nota: P-07 y P-09 son preguntas abiertas del documento 05 del proyecto; las demás derivan de observaciones de la revisión. La columna en color crema es para llenado de la DGIVA.</t>
         </is>
@@ -2786,8 +2760,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.6" right="0.6" top="0.7" bottom="0.7" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Auditoría de código y estilos sin restos (criterio 4); Versión 30
DEC-227: línea muerta, nombres de función repetidos, selectores
duplicados, colores fuera de :root, !important del modo revisión,
selectores por identificador y estilos en línea repetidos, corregidos.
La auditoría queda como batería 35, sobre prototipo y artefacto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWB8Tdi1QVG5m1csa2tJiV
</commit_message>
<xml_diff>
--- a/revision/Validacion-observaciones-DGIVA-v5.xlsx
+++ b/revision/Validacion-observaciones-DGIVA-v5.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Versión 29 · Validación DGIVA</t>
+          <t>Versión 30 · Validación DGIVA</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1875,7 @@
       <c r="J23" s="21" t="n"/>
       <c r="K23" s="21" t="n"/>
     </row>
-    <row r="24" ht="104" customHeight="1">
+    <row r="24" ht="65" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
           <t>OBS-0019</t>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="G24" s="19" t="inlineStr">
         <is>
-          <t>Se incorporó el contenido de la propuesta, en el registro de «tú» que usa todo el formulario: la Secretaría valora los hechos con el mismo rigor y el correo sirve para que la unidad administrativa que atiende la denuncia pueda ponerse en contacto. No se incluye el envío del informe de acciones por correo, porque el formulario no envía correos y no hay un plazo comprometido para informar. Después se simplificó (DEC-220): «Sí. Al final eliges presentarla anónima; sólo te pedimos un correo por si hay que aclarar algo. Se atiende con el mismo rigor.».</t>
+          <t>Se incorporó el contenido de la propuesta, en el registro de «tú» que usa todo el formulario. No se incluye el envío del informe de acciones por correo, porque el formulario no envía correos. Texto vigente: «Sí. Al final eliges presentarla anónima; sólo te pedimos un correo por si hay que aclarar algo. Se atiende con el mismo rigor, pero no se te notifica el resultado.».</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
         <is>
-          <t>DEC-195, DEC-220</t>
+          <t>DEC-195, DEC-220, DEC-226</t>
         </is>
       </c>
       <c r="I24" s="20" t="inlineStr">
@@ -2169,7 +2169,7 @@
       <c r="J29" s="21" t="n"/>
       <c r="K29" s="21" t="n"/>
     </row>
-    <row r="30" ht="65" customHeight="1">
+    <row r="30" ht="91" customHeight="1">
       <c r="A30" s="18" t="inlineStr">
         <is>
           <t>OBS-0025</t>
@@ -2202,12 +2202,12 @@
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
-          <t>La pregunta se conserva como opcional, con sus cuatro opciones. Al elegir «una persona» o «una empresa o negocio» ya no se abre ninguna pregunta adicional. «No lo sé» conserva un campo para describir lo observado, y «una autoridad de gobierno» sus campos, necesarios para la recomendación del artículo 331. Se atiende junto con OBS-0029.</t>
+          <t>La pregunta «¿Quién es responsable de los hechos?» se conserva, en lista desplegable, con «No lo sé» como respuesta para quien no lo sabe: no impide presentar la denuncia. Es obligatoria desde DEC-202, como quedó en el mapeo de campos que la DGIVA validó el 20 oct 2026. Al elegir «una persona» o «una empresa o negocio» no se abre ninguna pregunta adicional; «No lo sé» conserva un campo para describir lo observado, y «una autoridad de gobierno» pide el ámbito y cuál. Se atiende junto con OBS-0029.</t>
         </is>
       </c>
       <c r="H30" s="20" t="inlineStr">
         <is>
-          <t>DEC-193</t>
+          <t>DEC-193, DEC-202, DEC-226</t>
         </is>
       </c>
       <c r="I30" s="20" t="inlineStr">
@@ -2414,7 +2414,7 @@
       <c r="J34" s="21" t="n"/>
       <c r="K34" s="21" t="n"/>
     </row>
-    <row r="35" ht="30" customHeight="1">
+    <row r="35" ht="52" customHeight="1">
       <c r="A35" s="22" t="inlineStr">
         <is>
           <t>OBS-0030</t>
@@ -2447,12 +2447,12 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>La pregunta ya era opcional; ahora dice «(opcional)», como todos los campos no obligatorios.</t>
+          <t>«¿Ya reportaste estos hechos ante otra autoridad?» se contesta con sí o no y es obligatoria (DEC-202), como quedó en el mapeo de campos que la DGIVA validó el 20 oct 2026; el detalle «¿Ante quién, cuándo y qué respuesta recibiste?» es opcional.</t>
         </is>
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>DEC-191</t>
+          <t>DEC-191, DEC-202, DEC-226</t>
         </is>
       </c>
       <c r="I35" s="24" t="inlineStr">

</xml_diff>